<commit_message>
Atualização automática: Ranking CNB 2026
</commit_message>
<xml_diff>
--- a/Ranking_CNB_2026.xlsx
+++ b/Ranking_CNB_2026.xlsx
@@ -458,12 +458,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2.048,3 km</t>
+          <t>2.073,2 km</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>32.179 m</t>
+          <t>32.404 m</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -478,16 +478,16 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>888,9 km</t>
+          <t>904,0 km</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>9.359 m</t>
+          <t>9.497 m</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4">
@@ -518,16 +518,16 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>257,2 km</t>
+          <t>260,1 km</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2.826 m</t>
+          <t>2.862 m</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>